<commit_message>
migration updated including nsonepal
</commit_message>
<xml_diff>
--- a/migration/tables.xlsx
+++ b/migration/tables.xlsx
@@ -1,33 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\migration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D521F42A-86A8-4226-835A-041BDABAC706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA42964-9E65-4F42-9B85-7EF7703DD936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5100" yWindow="3015" windowWidth="15375" windowHeight="7785" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Reasons for leaving origin" sheetId="1" r:id="rId1"/>
     <sheet name="Distribution of Households" sheetId="2" r:id="rId2"/>
     <sheet name="Satisfaction" sheetId="3" r:id="rId3"/>
+    <sheet name="Datewise migrants no." sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
   <si>
     <t>2. Table No. 5.1.1: Distribution of Reasons for Leaving Place of Origin</t>
   </si>
@@ -103,12 +114,45 @@
   <si>
     <t>Same as before</t>
   </si>
+  <si>
+    <t>Years</t>
+  </si>
+  <si>
+    <t>Households</t>
+  </si>
+  <si>
+    <t>Ethnicity</t>
+  </si>
+  <si>
+    <t>No. of households</t>
+  </si>
+  <si>
+    <t>Percent</t>
+  </si>
+  <si>
+    <t>Brahmin</t>
+  </si>
+  <si>
+    <t>Chettri</t>
+  </si>
+  <si>
+    <t>Gurung</t>
+  </si>
+  <si>
+    <t>Kami</t>
+  </si>
+  <si>
+    <t>Sarki</t>
+  </si>
+  <si>
+    <t>Others</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -142,6 +186,14 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -157,7 +209,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -217,11 +269,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -250,6 +317,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -882,6 +952,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-9E8E-4A8C-BC1B-F97AD8813454}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -897,6 +972,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-9E8E-4A8C-BC1B-F97AD8813454}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -912,6 +992,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-9E8E-4A8C-BC1B-F97AD8813454}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -927,6 +1012,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-9E8E-4A8C-BC1B-F97AD8813454}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="4"/>
@@ -942,6 +1032,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-9E8E-4A8C-BC1B-F97AD8813454}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="5"/>
@@ -957,6 +1052,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000B-9E8E-4A8C-BC1B-F97AD8813454}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="6"/>
@@ -974,6 +1074,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000D-9E8E-4A8C-BC1B-F97AD8813454}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="7"/>
@@ -991,6 +1096,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000F-9E8E-4A8C-BC1B-F97AD8813454}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
@@ -6957,4 +7067,178 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C959D8AD-7ECD-4483-A446-BE63C69CCCAE}">
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="11">
+        <v>2083</v>
+      </c>
+      <c r="B2" s="11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="11">
+        <v>2082</v>
+      </c>
+      <c r="B3" s="11">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="11">
+        <v>2081</v>
+      </c>
+      <c r="B4" s="11">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="11">
+        <v>2080</v>
+      </c>
+      <c r="B5" s="11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="11">
+        <v>2079</v>
+      </c>
+      <c r="B6" s="11">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="11">
+        <v>2078</v>
+      </c>
+      <c r="B7" s="11">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="11">
+        <v>2077</v>
+      </c>
+      <c r="B8" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="11">
+        <v>2076</v>
+      </c>
+      <c r="B9" s="11">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="11">
+        <v>2075</v>
+      </c>
+      <c r="B10" s="11">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="11">
+        <v>2074</v>
+      </c>
+      <c r="B11" s="11">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0507400-295F-49FC-B948-B908FD858BD5}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
migration continue and saruwa edited
</commit_message>
<xml_diff>
--- a/migration/tables.xlsx
+++ b/migration/tables.xlsx
@@ -1,23 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\migration\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\082_083\ward1\migration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AA42964-9E65-4F42-9B85-7EF7703DD936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC567BF5-17C6-4CE2-81CB-335F8278E273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5100" yWindow="3015" windowWidth="15375" windowHeight="7785" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11184" yWindow="0" windowWidth="11880" windowHeight="12360" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Reasons for leaving origin" sheetId="1" r:id="rId1"/>
     <sheet name="Distribution of Households" sheetId="2" r:id="rId2"/>
     <sheet name="Satisfaction" sheetId="3" r:id="rId3"/>
     <sheet name="Datewise migrants no." sheetId="4" r:id="rId4"/>
-    <sheet name="Sheet2" sheetId="5" r:id="rId5"/>
+    <sheet name="Literacy status" sheetId="6" r:id="rId5"/>
+    <sheet name="Ethnicity" sheetId="5" r:id="rId6"/>
+    <sheet name="Religion" sheetId="7" r:id="rId7"/>
+    <sheet name="Land holdings" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,6 +34,8 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -38,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="54">
   <si>
     <t>2. Table No. 5.1.1: Distribution of Reasons for Leaving Place of Origin</t>
   </si>
@@ -136,16 +141,70 @@
     <t>Chettri</t>
   </si>
   <si>
-    <t>Gurung</t>
+    <t>Others</t>
   </si>
   <si>
-    <t>Kami</t>
+    <t>Literacy Status</t>
   </si>
   <si>
-    <t>Sarki</t>
+    <t>Sex</t>
   </si>
   <si>
-    <t>Others</t>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No. </t>
+  </si>
+  <si>
+    <t>Literate</t>
+  </si>
+  <si>
+    <t>Illiterate</t>
+  </si>
+  <si>
+    <t>Janajati</t>
+  </si>
+  <si>
+    <t>Dalit</t>
+  </si>
+  <si>
+    <t>Religion</t>
+  </si>
+  <si>
+    <t>Hindu</t>
+  </si>
+  <si>
+    <t>Buddhist</t>
+  </si>
+  <si>
+    <t>Muslim</t>
+  </si>
+  <si>
+    <t>Christian</t>
+  </si>
+  <si>
+    <t>Size of Land Holding</t>
+  </si>
+  <si>
+    <t>Percentage (%)</t>
+  </si>
+  <si>
+    <t>Ropani</t>
+  </si>
+  <si>
+    <t>Aana</t>
+  </si>
+  <si>
+    <t>Paisa</t>
+  </si>
+  <si>
+    <t>Daam</t>
+  </si>
+  <si>
+    <t>-</t>
   </si>
 </sst>
 </file>
@@ -209,7 +268,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -284,11 +343,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -311,15 +379,28 @@
     <xf numFmtId="10" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2920,6 +3001,563 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Male</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Literacy status'!$I$3:$J$3</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Literate</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Illiterate</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Literacy status'!$I$4:$I$5</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>93.75</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6.25</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C491-4805-9B7F-E54A41F0E2D7}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Female</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Literacy status'!$I$3:$J$3</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Literate</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Illiterate</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Literacy status'!$J$4:$J$5</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>62.893081761006286</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>37.106918238993707</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-C491-4805-9B7F-E54A41F0E2D7}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="199"/>
+        <c:axId val="1948943712"/>
+        <c:axId val="1948944960"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1948943712"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" b="1" cap="none" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Literacy Status</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1948944960"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1948944960"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:minorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="5000"/>
+                  <a:lumOff val="95000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" b="1" cap="none" normalizeH="0" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Percent</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1948943712"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -3160,6 +3798,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors7.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -6212,6 +6890,506 @@
         <a:noFill/>
       </a:ln>
     </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style7.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="212">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200" cap="all"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="38100" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="8"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="major">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="2000" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
   </cs:wall>
 </cs:chartStyle>
 </file>
@@ -6447,6 +7625,47 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>350520</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>102870</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>525780</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0500-000006000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -6711,41 +7930,41 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.3">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
     </row>
-    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
     </row>
-    <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -6756,7 +7975,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
@@ -6767,7 +7986,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
@@ -6778,7 +7997,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
@@ -6789,7 +8008,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
@@ -6800,7 +8019,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
@@ -6811,7 +8030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
@@ -6822,7 +8041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>11</v>
       </c>
@@ -6833,7 +8052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>12</v>
       </c>
@@ -6855,49 +8074,49 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4023F4C3-8104-49AA-9B04-0E3072F18EBB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.3">
+      <c r="A1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>15</v>
       </c>
@@ -6908,7 +8127,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>16</v>
       </c>
@@ -6919,7 +8138,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>17</v>
       </c>
@@ -6930,7 +8149,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>18</v>
       </c>
@@ -6941,7 +8160,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -6963,48 +8182,48 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C17A5493-1664-4BB0-9A54-26F7CA5546B7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.140625" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.3">
+      <c r="A1" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
     </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
     </row>
-    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>21</v>
       </c>
@@ -7015,7 +8234,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -7026,7 +8245,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>23</v>
       </c>
@@ -7037,7 +8256,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>24</v>
       </c>
@@ -7048,7 +8267,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -7070,98 +8289,98 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C959D8AD-7ECD-4483-A446-BE63C69CCCAE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="8" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="11">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="9">
         <v>2083</v>
       </c>
-      <c r="B2" s="11">
+      <c r="B2" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="11">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
         <v>2082</v>
       </c>
-      <c r="B3" s="11">
+      <c r="B3" s="9">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="11">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
         <v>2081</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="9">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="11">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="9">
         <v>2080</v>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="9">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="11">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="9">
         <v>2079</v>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="9">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="11">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="9">
         <v>2078</v>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="9">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="11">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="9">
         <v>2077</v>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="9">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="11">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="9">
         <v>2076</v>
       </c>
-      <c r="B9" s="11">
+      <c r="B9" s="9">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="11">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="9">
         <v>2075</v>
       </c>
-      <c r="B10" s="11">
+      <c r="B10" s="9">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="11">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="9">
         <v>2074</v>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="9">
         <v>9</v>
       </c>
     </row>
@@ -7171,72 +8390,453 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0507400-295F-49FC-B948-B908FD858BD5}">
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:J6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="15"/>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2" s="15"/>
+      <c r="B2" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" s="14"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3" s="15"/>
+      <c r="B3" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="10">
+        <f>164+1</f>
+        <v>165</v>
+      </c>
+      <c r="C4" s="12">
+        <f>B4/B6*100</f>
+        <v>93.75</v>
+      </c>
+      <c r="D4" s="10">
+        <f>99+1</f>
+        <v>100</v>
+      </c>
+      <c r="E4" s="12">
+        <f>D4/D6*100</f>
+        <v>62.893081761006286</v>
+      </c>
+      <c r="F4" s="10">
+        <f>B4+D4</f>
+        <v>265</v>
+      </c>
+      <c r="G4" s="12">
+        <f>F4/F6*100</f>
+        <v>79.104477611940297</v>
+      </c>
+      <c r="I4" s="12">
+        <v>93.75</v>
+      </c>
+      <c r="J4" s="12">
+        <v>62.893081761006286</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" s="10">
+        <v>11</v>
+      </c>
+      <c r="C5" s="12">
+        <f>B5/B6*100</f>
+        <v>6.25</v>
+      </c>
+      <c r="D5" s="10">
+        <f>58+1</f>
+        <v>59</v>
+      </c>
+      <c r="E5" s="12">
+        <f>D5/D6*100</f>
+        <v>37.106918238993707</v>
+      </c>
+      <c r="F5" s="10">
+        <f>B5+D5</f>
+        <v>70</v>
+      </c>
+      <c r="G5" s="12">
+        <f>F5/F6*100</f>
+        <v>20.8955223880597</v>
+      </c>
+      <c r="I5" s="12">
+        <v>6.25</v>
+      </c>
+      <c r="J5" s="12">
+        <v>37.106918238993707</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="10">
+        <f>SUM(B4:B5)</f>
+        <v>176</v>
+      </c>
+      <c r="C6" s="10">
+        <f t="shared" ref="C6:G6" si="0">SUM(C4:C5)</f>
+        <v>100</v>
+      </c>
+      <c r="D6" s="10">
+        <f t="shared" si="0"/>
+        <v>159</v>
+      </c>
+      <c r="E6" s="10">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="F6" s="10">
+        <f t="shared" si="0"/>
+        <v>335</v>
+      </c>
+      <c r="G6" s="10">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F1:G2"/>
+    <mergeCell ref="A1:A3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
+      <c r="B2" s="10">
+        <v>31</v>
+      </c>
+      <c r="C2" s="12">
+        <f>B2/B6*100</f>
+        <v>34.831460674157306</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
+      <c r="B3" s="10">
+        <v>25</v>
+      </c>
+      <c r="C3" s="12">
+        <f>B3/B6*100</f>
+        <v>28.08988764044944</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="10">
+        <v>25</v>
+      </c>
+      <c r="C4" s="12">
+        <f>B4/B6*100</f>
+        <v>28.08988764044944</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="10">
+        <v>8</v>
+      </c>
+      <c r="C5" s="12">
+        <f>B5/B6*100</f>
+        <v>8.9887640449438209</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="10">
+        <f>SUM(B2:B5)</f>
+        <v>89</v>
+      </c>
+      <c r="C6" s="10">
+        <f>SUM(C2:C5)</f>
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17375082-251D-4B38-966E-F88F9E772705}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="10">
+        <v>31</v>
+      </c>
+      <c r="C2" s="12">
+        <f>B2/B7*100</f>
+        <v>34.831460674157306</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="10">
+        <v>25</v>
+      </c>
+      <c r="C3" s="12">
+        <f>B3/B7*100</f>
+        <v>28.08988764044944</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="10">
+        <v>25</v>
+      </c>
+      <c r="C4" s="12">
+        <f>B4/B7*100</f>
+        <v>28.08988764044944</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="10">
+        <v>8</v>
+      </c>
+      <c r="C5" s="12">
+        <f>B5/B7*100</f>
+        <v>8.9887640449438209</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" s="12"/>
+      <c r="B6" s="10"/>
       <c r="C6" s="12"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="10">
+        <f>SUM(B2:B5)</f>
+        <v>89</v>
+      </c>
+      <c r="C7" s="10">
+        <f>SUM(C2:C5)</f>
+        <v>100</v>
+      </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{313C3968-0C2C-495D-B103-63BB836806C3}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B2" s="10">
+        <v>13</v>
+      </c>
+      <c r="C2" s="12">
+        <f>B2/$B$7*100</f>
+        <v>14.606741573033707</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="10">
+        <v>52</v>
+      </c>
+      <c r="C3" s="12">
+        <f t="shared" ref="C3:C6" si="0">B3/$B$7*100</f>
+        <v>58.426966292134829</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" s="10">
+        <v>0</v>
+      </c>
+      <c r="C4" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="10">
+        <v>0</v>
+      </c>
+      <c r="C5" s="12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="10">
+        <v>24</v>
+      </c>
+      <c r="C6" s="12">
+        <f t="shared" si="0"/>
+        <v>26.966292134831459</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
+      <c r="B7" s="10">
+        <f>SUM(B2:B6)</f>
+        <v>89</v>
+      </c>
+      <c r="C7" s="10">
+        <f>SUM(C2:C6)</f>
+        <v>100</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
migration water source and age group done
</commit_message>
<xml_diff>
--- a/migration/tables.xlsx
+++ b/migration/tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\082_083\ward1\migration\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\migration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC567BF5-17C6-4CE2-81CB-335F8278E273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F9FBE09-9D85-4FAF-B6B7-2FD3E977FF05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11184" yWindow="0" windowWidth="11880" windowHeight="12360" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Reasons for leaving origin" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,8 @@
     <sheet name="Ethnicity" sheetId="5" r:id="rId6"/>
     <sheet name="Religion" sheetId="7" r:id="rId7"/>
     <sheet name="Land holdings" sheetId="8" r:id="rId8"/>
+    <sheet name="Water source" sheetId="9" r:id="rId9"/>
+    <sheet name="5yrs age group" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,8 +36,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="74">
   <si>
     <t>2. Table No. 5.1.1: Distribution of Reasons for Leaving Place of Origin</t>
   </si>
@@ -204,7 +204,67 @@
     <t>Daam</t>
   </si>
   <si>
-    <t>-</t>
+    <t>No land</t>
+  </si>
+  <si>
+    <t>Sources of Water</t>
+  </si>
+  <si>
+    <t>Piped</t>
+  </si>
+  <si>
+    <t>Well</t>
+  </si>
+  <si>
+    <t>Boring</t>
+  </si>
+  <si>
+    <t>0-4</t>
+  </si>
+  <si>
+    <t>5-9</t>
+  </si>
+  <si>
+    <t>10-14</t>
+  </si>
+  <si>
+    <t>15-19</t>
+  </si>
+  <si>
+    <t>20-24</t>
+  </si>
+  <si>
+    <t>25-29</t>
+  </si>
+  <si>
+    <t>30-34</t>
+  </si>
+  <si>
+    <t>35-39</t>
+  </si>
+  <si>
+    <t>40-44</t>
+  </si>
+  <si>
+    <t>45-49</t>
+  </si>
+  <si>
+    <t>50-54</t>
+  </si>
+  <si>
+    <t>54-59</t>
+  </si>
+  <si>
+    <t>60-64</t>
+  </si>
+  <si>
+    <t>65+</t>
+  </si>
+  <si>
+    <t>Sex of the Migrants</t>
+  </si>
+  <si>
+    <t>Age Group</t>
   </si>
 </sst>
 </file>
@@ -268,7 +328,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -343,20 +403,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -380,14 +431,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -395,12 +448,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -924,6 +980,354 @@
           <a:lumOff val="85000"/>
         </a:schemeClr>
       </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:view3D>
+      <c:rotX val="30"/>
+      <c:rotY val="0"/>
+      <c:depthPercent val="100"/>
+      <c:rAngAx val="0"/>
+    </c:view3D>
+    <c:floor>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:floor>
+    <c:sideWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:sideWall>
+    <c:backWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:backWall>
+    <c:plotArea>
+      <c:layout/>
+      <c:pie3DChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:pattFill prst="pct5">
+              <a:fgClr>
+                <a:schemeClr val="tx1"/>
+              </a:fgClr>
+              <a:bgClr>
+                <a:schemeClr val="bg1"/>
+              </a:bgClr>
+            </a:pattFill>
+            <a:ln>
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="dashHorz">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst>
+                <a:outerShdw blurRad="50800" dist="38100" dir="2700000" algn="tl" rotWithShape="0">
+                  <a:schemeClr val="bg1">
+                    <a:lumMod val="65000"/>
+                    <a:alpha val="40000"/>
+                  </a:schemeClr>
+                </a:outerShdw>
+              </a:effectLst>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-71A5-4D71-81F3-625022BF6838}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="ltDnDiag">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-71A5-4D71-81F3-625022BF6838}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="pct5">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-71A5-4D71-81F3-625022BF6838}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:gradFill flip="none" rotWithShape="1">
+                <a:gsLst>
+                  <a:gs pos="0">
+                    <a:schemeClr val="accent3">
+                      <a:lumMod val="5000"/>
+                      <a:lumOff val="95000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="74000">
+                    <a:schemeClr val="accent3">
+                      <a:lumMod val="45000"/>
+                      <a:lumOff val="55000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="83000">
+                    <a:schemeClr val="accent3">
+                      <a:lumMod val="45000"/>
+                      <a:lumOff val="55000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="accent3">
+                      <a:lumMod val="30000"/>
+                      <a:lumOff val="70000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="5400000" scaled="1"/>
+                <a:tileRect/>
+              </a:gradFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="1"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="35000"/>
+                      <a:lumOff val="65000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:round/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Water source'!$F$2:$F$4</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Piped</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Boring</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Well</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Water source'!$G$2:$G$4</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>6.7415730337078648</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>39.325842696629216</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>53.932584269662918</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-71A5-4D71-81F3-625022BF6838}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="1"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+      </c:pie3DChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:noFill/>
       <a:round/>
     </a:ln>
     <a:effectLst/>
@@ -3029,11 +3433,11 @@
             <c:v>Male</c:v>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
+            <a:noFill/>
             <a:ln>
-              <a:noFill/>
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
@@ -3096,7 +3500,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Literacy status'!$I$3:$J$3</c:f>
+              <c:f>'Literacy status'!$J$3:$K$3</c:f>
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
@@ -3110,15 +3514,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Literacy status'!$I$4:$I$5</c:f>
+              <c:f>'Literacy status'!$J$4:$J$5</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>93.75</c:v>
+                  <c:v>93.714285714285722</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.25</c:v>
+                  <c:v>6.2857142857142865</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3136,11 +3540,18 @@
             <c:v>Female</c:v>
           </c:tx>
           <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent2"/>
-            </a:solidFill>
+            <a:pattFill prst="dashVert">
+              <a:fgClr>
+                <a:schemeClr val="tx1"/>
+              </a:fgClr>
+              <a:bgClr>
+                <a:schemeClr val="bg1"/>
+              </a:bgClr>
+            </a:pattFill>
             <a:ln>
-              <a:noFill/>
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
@@ -3204,7 +3615,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>'Literacy status'!$I$3:$J$3</c:f>
+              <c:f>'Literacy status'!$J$3:$K$3</c:f>
               <c:strCache>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
@@ -3218,15 +3629,15 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'Literacy status'!$J$4:$J$5</c:f>
+              <c:f>'Literacy status'!$K$4:$K$5</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>62.893081761006286</c:v>
+                  <c:v>66.875</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>37.106918238993707</c:v>
+                  <c:v>33.125</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3558,7 +3969,795 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:view3D>
+      <c:rotX val="30"/>
+      <c:rotY val="0"/>
+      <c:depthPercent val="100"/>
+      <c:rAngAx val="0"/>
+    </c:view3D>
+    <c:floor>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:floor>
+    <c:sideWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:sideWall>
+    <c:backWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:backWall>
+    <c:plotArea>
+      <c:layout/>
+      <c:pie3DChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln>
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="pct5">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d>
+                <a:contourClr>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-0DC4-4BD0-BCA4-3F70E80E4AE5}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="weave">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d>
+                <a:contourClr>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000004-0DC4-4BD0-BCA4-3F70E80E4AE5}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="dotDmnd">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d>
+                <a:contourClr>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-0DC4-4BD0-BCA4-3F70E80E4AE5}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="ltUpDiag">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d>
+                <a:contourClr>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-0DC4-4BD0-BCA4-3F70E80E4AE5}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:gradFill>
+                <a:gsLst>
+                  <a:gs pos="0">
+                    <a:schemeClr val="accent1">
+                      <a:lumMod val="5000"/>
+                      <a:lumOff val="95000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="74000">
+                    <a:schemeClr val="accent1">
+                      <a:lumMod val="45000"/>
+                      <a:lumOff val="55000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="83000">
+                    <a:schemeClr val="accent1">
+                      <a:lumMod val="45000"/>
+                      <a:lumOff val="55000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                  <a:gs pos="100000">
+                    <a:schemeClr val="accent1">
+                      <a:lumMod val="30000"/>
+                      <a:lumOff val="70000"/>
+                    </a:schemeClr>
+                  </a:gs>
+                </a:gsLst>
+                <a:lin ang="5400000" scaled="1"/>
+              </a:gradFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx2"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="1"/>
+            <c:leaderLines>
+              <c:spPr>
+                <a:ln w="9525">
+                  <a:solidFill>
+                    <a:schemeClr val="tx2">
+                      <a:lumMod val="35000"/>
+                      <a:lumOff val="65000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:leaderLines>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Ethnicity!$F$2:$F$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Brahmin</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Chettri</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Janajati</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Dalit</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Ethnicity!$G$2:$G$5</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>34.831460674157306</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>28.08988764044944</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>28.08988764044944</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.9887640449438209</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-0DC4-4BD0-BCA4-3F70E80E4AE5}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+      </c:pie3DChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx2"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx2">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="pct20">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-AE78-4BA4-AC36-CAC6F298C969}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="pct20">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000004-AE78-4BA4-AC36-CAC6F298C969}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="pct20">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000006-AE78-4BA4-AC36-CAC6F298C969}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:pattFill prst="pct20">
+                <a:fgClr>
+                  <a:schemeClr val="tx1"/>
+                </a:fgClr>
+                <a:bgClr>
+                  <a:schemeClr val="bg1"/>
+                </a:bgClr>
+              </a:pattFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-AE78-4BA4-AC36-CAC6F298C969}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>Religion!$F$2:$F$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>Hindu</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Buddhist</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Muslim</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Christian</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Religion!$G$2:$G$5</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>34.831460674157306</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>28.08988764044944</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>28.08988764044944</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.9887640449438209</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-AE78-4BA4-AC36-CAC6F298C969}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="356970591"/>
+        <c:axId val="251624399"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="356970591"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="251624399"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="251624399"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="356970591"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors10.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -3838,6 +5037,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors8.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors9.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -4309,6 +5588,525 @@
             <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style10.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="262">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -7390,6 +9188,977 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="dk1"/>
     </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style8.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="266">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" b="1" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk2">
+        <a:lumMod val="75000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="31750" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="12700">
+        <a:solidFill>
+          <a:schemeClr val="lt2"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="2"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="1600" b="1" kern="1200"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx2"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style9.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
   </cs:wall>
 </cs:chartStyle>
 </file>
@@ -7666,6 +10435,129 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>80962</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BFC834FE-EB00-B6DE-B2AC-977A6245A4B8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>300037</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>52387</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>604837</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>128587</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB882F85-A674-F707-3722-99B1F7F8EDE6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>547687</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>52387</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>242887</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>128587</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BBE0CE10-00BA-C677-EBE8-7A4E78C2C427}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -7930,41 +10822,41 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:9" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
     </row>
-    <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
     </row>
-    <row r="3" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -7975,7 +10867,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
@@ -7986,7 +10878,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
@@ -7997,7 +10889,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
@@ -8008,7 +10900,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
@@ -8019,7 +10911,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
@@ -8030,7 +10922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
@@ -8041,7 +10933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>11</v>
       </c>
@@ -8052,7 +10944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>12</v>
       </c>
@@ -8073,50 +10965,554 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4681C5CD-AD1E-47C1-9DD5-E5803D1EB1C3}">
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="15"/>
+      <c r="B2" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="20">
+        <v>6</v>
+      </c>
+      <c r="C3" s="11">
+        <f>B3/$B$17*100</f>
+        <v>3.3149171270718232</v>
+      </c>
+      <c r="D3" s="20">
+        <v>4</v>
+      </c>
+      <c r="E3" s="11">
+        <f>D3/$D$17*100</f>
+        <v>2.4390243902439024</v>
+      </c>
+      <c r="F3" s="20">
+        <v>10</v>
+      </c>
+      <c r="G3" s="11">
+        <f>F3/$F$17*100</f>
+        <v>2.8985507246376812</v>
+      </c>
+      <c r="I3" s="17">
+        <f>(C3+E3)/2</f>
+        <v>2.8769707586578628</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B4" s="20">
+        <v>7</v>
+      </c>
+      <c r="C4" s="11">
+        <f t="shared" ref="C4:C17" si="0">B4/$B$17*100</f>
+        <v>3.867403314917127</v>
+      </c>
+      <c r="D4" s="20">
+        <v>4</v>
+      </c>
+      <c r="E4" s="11">
+        <f t="shared" ref="E4:E16" si="1">D4/$D$17*100</f>
+        <v>2.4390243902439024</v>
+      </c>
+      <c r="F4" s="20">
+        <v>11</v>
+      </c>
+      <c r="G4" s="11">
+        <f t="shared" ref="G4:G17" si="2">F4/$F$17*100</f>
+        <v>3.1884057971014492</v>
+      </c>
+      <c r="I4" s="17">
+        <f t="shared" ref="I4:I16" si="3">(C4+E4)/2</f>
+        <v>3.1532138525805147</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="20">
+        <v>14</v>
+      </c>
+      <c r="C5" s="11">
+        <f t="shared" si="0"/>
+        <v>7.7348066298342539</v>
+      </c>
+      <c r="D5" s="20">
+        <v>11</v>
+      </c>
+      <c r="E5" s="11">
+        <f t="shared" si="1"/>
+        <v>6.7073170731707323</v>
+      </c>
+      <c r="F5" s="20">
+        <v>25</v>
+      </c>
+      <c r="G5" s="11">
+        <f t="shared" si="2"/>
+        <v>7.2463768115942031</v>
+      </c>
+      <c r="I5" s="17">
+        <f t="shared" si="3"/>
+        <v>7.2210618515024931</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="20">
+        <v>7</v>
+      </c>
+      <c r="C6" s="11">
+        <f t="shared" si="0"/>
+        <v>3.867403314917127</v>
+      </c>
+      <c r="D6" s="20">
+        <v>10</v>
+      </c>
+      <c r="E6" s="11">
+        <f t="shared" si="1"/>
+        <v>6.0975609756097562</v>
+      </c>
+      <c r="F6" s="20">
+        <v>17</v>
+      </c>
+      <c r="G6" s="11">
+        <f t="shared" si="2"/>
+        <v>4.9275362318840585</v>
+      </c>
+      <c r="I6" s="17">
+        <f t="shared" si="3"/>
+        <v>4.9824821452634414</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="20">
+        <v>20</v>
+      </c>
+      <c r="C7" s="11">
+        <f t="shared" si="0"/>
+        <v>11.049723756906078</v>
+      </c>
+      <c r="D7" s="20">
+        <v>13</v>
+      </c>
+      <c r="E7" s="11">
+        <f t="shared" si="1"/>
+        <v>7.9268292682926829</v>
+      </c>
+      <c r="F7" s="20">
+        <v>33</v>
+      </c>
+      <c r="G7" s="11">
+        <f t="shared" si="2"/>
+        <v>9.5652173913043477</v>
+      </c>
+      <c r="I7" s="17">
+        <f t="shared" si="3"/>
+        <v>9.4882765125993807</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B8" s="20">
+        <v>15</v>
+      </c>
+      <c r="C8" s="11">
+        <f t="shared" si="0"/>
+        <v>8.2872928176795568</v>
+      </c>
+      <c r="D8" s="20">
+        <v>15</v>
+      </c>
+      <c r="E8" s="11">
+        <f t="shared" si="1"/>
+        <v>9.1463414634146343</v>
+      </c>
+      <c r="F8" s="20">
+        <v>30</v>
+      </c>
+      <c r="G8" s="11">
+        <f t="shared" si="2"/>
+        <v>8.695652173913043</v>
+      </c>
+      <c r="I8" s="17">
+        <f t="shared" si="3"/>
+        <v>8.7168171405470964</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="B9" s="20">
+        <v>19</v>
+      </c>
+      <c r="C9" s="11">
+        <f t="shared" si="0"/>
+        <v>10.497237569060774</v>
+      </c>
+      <c r="D9" s="20">
+        <v>17</v>
+      </c>
+      <c r="E9" s="11">
+        <f t="shared" si="1"/>
+        <v>10.365853658536585</v>
+      </c>
+      <c r="F9" s="20">
+        <v>36</v>
+      </c>
+      <c r="G9" s="11">
+        <f t="shared" si="2"/>
+        <v>10.434782608695652</v>
+      </c>
+      <c r="I9" s="17">
+        <f t="shared" si="3"/>
+        <v>10.431545613798679</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="20">
+        <v>12</v>
+      </c>
+      <c r="C10" s="11">
+        <f t="shared" si="0"/>
+        <v>6.6298342541436464</v>
+      </c>
+      <c r="D10" s="20">
+        <v>17</v>
+      </c>
+      <c r="E10" s="11">
+        <f t="shared" si="1"/>
+        <v>10.365853658536585</v>
+      </c>
+      <c r="F10" s="20">
+        <v>29</v>
+      </c>
+      <c r="G10" s="11">
+        <f t="shared" si="2"/>
+        <v>8.4057971014492754</v>
+      </c>
+      <c r="I10" s="17">
+        <f t="shared" si="3"/>
+        <v>8.497843956340116</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="20">
+        <v>12</v>
+      </c>
+      <c r="C11" s="11">
+        <f t="shared" si="0"/>
+        <v>6.6298342541436464</v>
+      </c>
+      <c r="D11" s="20">
+        <v>21</v>
+      </c>
+      <c r="E11" s="11">
+        <f t="shared" si="1"/>
+        <v>12.804878048780488</v>
+      </c>
+      <c r="F11" s="20">
+        <v>33</v>
+      </c>
+      <c r="G11" s="11">
+        <f t="shared" si="2"/>
+        <v>9.5652173913043477</v>
+      </c>
+      <c r="I11" s="17">
+        <f t="shared" si="3"/>
+        <v>9.7173561514620665</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="20">
+        <v>19</v>
+      </c>
+      <c r="C12" s="11">
+        <f t="shared" si="0"/>
+        <v>10.497237569060774</v>
+      </c>
+      <c r="D12" s="20">
+        <v>8</v>
+      </c>
+      <c r="E12" s="11">
+        <f t="shared" si="1"/>
+        <v>4.8780487804878048</v>
+      </c>
+      <c r="F12" s="20">
+        <v>27</v>
+      </c>
+      <c r="G12" s="11">
+        <f t="shared" si="2"/>
+        <v>7.8260869565217401</v>
+      </c>
+      <c r="I12" s="17">
+        <f t="shared" si="3"/>
+        <v>7.6876431747742888</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="20">
+        <v>12</v>
+      </c>
+      <c r="C13" s="11">
+        <f t="shared" si="0"/>
+        <v>6.6298342541436464</v>
+      </c>
+      <c r="D13" s="20">
+        <v>18</v>
+      </c>
+      <c r="E13" s="11">
+        <f t="shared" si="1"/>
+        <v>10.975609756097562</v>
+      </c>
+      <c r="F13" s="20">
+        <v>30</v>
+      </c>
+      <c r="G13" s="11">
+        <f t="shared" si="2"/>
+        <v>8.695652173913043</v>
+      </c>
+      <c r="I13" s="17">
+        <f t="shared" si="3"/>
+        <v>8.8027220051206037</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="20">
+        <v>16</v>
+      </c>
+      <c r="C14" s="11">
+        <f t="shared" si="0"/>
+        <v>8.8397790055248606</v>
+      </c>
+      <c r="D14" s="20">
+        <v>12</v>
+      </c>
+      <c r="E14" s="11">
+        <f t="shared" si="1"/>
+        <v>7.3170731707317067</v>
+      </c>
+      <c r="F14" s="20">
+        <v>28</v>
+      </c>
+      <c r="G14" s="11">
+        <f t="shared" si="2"/>
+        <v>8.115942028985506</v>
+      </c>
+      <c r="I14" s="17">
+        <f t="shared" si="3"/>
+        <v>8.0784260881282837</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="20">
+        <v>10</v>
+      </c>
+      <c r="C15" s="11">
+        <f t="shared" si="0"/>
+        <v>5.5248618784530388</v>
+      </c>
+      <c r="D15" s="20">
+        <v>3</v>
+      </c>
+      <c r="E15" s="11">
+        <f t="shared" si="1"/>
+        <v>1.8292682926829267</v>
+      </c>
+      <c r="F15" s="20">
+        <v>13</v>
+      </c>
+      <c r="G15" s="11">
+        <f t="shared" si="2"/>
+        <v>3.7681159420289858</v>
+      </c>
+      <c r="I15" s="17">
+        <f t="shared" si="3"/>
+        <v>3.6770650855679827</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="20">
+        <v>12</v>
+      </c>
+      <c r="C16" s="11">
+        <f t="shared" si="0"/>
+        <v>6.6298342541436464</v>
+      </c>
+      <c r="D16" s="20">
+        <v>11</v>
+      </c>
+      <c r="E16" s="11">
+        <f t="shared" si="1"/>
+        <v>6.7073170731707323</v>
+      </c>
+      <c r="F16" s="20">
+        <v>23</v>
+      </c>
+      <c r="G16" s="11">
+        <f t="shared" si="2"/>
+        <v>6.666666666666667</v>
+      </c>
+      <c r="I16" s="17">
+        <f t="shared" si="3"/>
+        <v>6.6685756636571893</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="20">
+        <v>181</v>
+      </c>
+      <c r="C17" s="11">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+      <c r="D17" s="20">
+        <v>164</v>
+      </c>
+      <c r="E17" s="11">
+        <f>D17/$D$17*100</f>
+        <v>100</v>
+      </c>
+      <c r="F17" s="20">
+        <v>345</v>
+      </c>
+      <c r="G17" s="11">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:12" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:12" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>15</v>
       </c>
@@ -8127,7 +11523,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>16</v>
       </c>
@@ -8138,7 +11534,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>17</v>
       </c>
@@ -8149,7 +11545,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>18</v>
       </c>
@@ -8160,7 +11556,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -8184,46 +11580,46 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
     </row>
-    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13"/>
+      <c r="I2" s="13"/>
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
     </row>
-    <row r="3" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>21</v>
       </c>
@@ -8234,7 +11630,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -8245,7 +11641,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>23</v>
       </c>
@@ -8256,7 +11652,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>24</v>
       </c>
@@ -8267,7 +11663,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -8290,13 +11686,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>25</v>
       </c>
@@ -8304,7 +11700,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>2083</v>
       </c>
@@ -8312,7 +11708,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="9">
         <v>2082</v>
       </c>
@@ -8320,7 +11716,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>2081</v>
       </c>
@@ -8328,7 +11724,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
         <v>2080</v>
       </c>
@@ -8336,7 +11732,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>2079</v>
       </c>
@@ -8344,7 +11740,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
         <v>2078</v>
       </c>
@@ -8352,7 +11748,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
         <v>2077</v>
       </c>
@@ -8360,7 +11756,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
         <v>2076</v>
       </c>
@@ -8368,7 +11764,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
         <v>2075</v>
       </c>
@@ -8376,12 +11772,21 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
         <v>2074</v>
       </c>
       <c r="B11" s="9">
         <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="9">
+        <f>SUM(B2:B11)</f>
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -8391,10 +11796,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
         <v>33</v>
       </c>
@@ -8409,7 +11814,7 @@
       </c>
       <c r="G1" s="15"/>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="15"/>
       <c r="B2" s="14" t="s">
         <v>36</v>
@@ -8422,127 +11827,130 @@
       <c r="F2" s="15"/>
       <c r="G2" s="15"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="15"/>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="G3" s="11" t="s">
+      <c r="G3" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="J3" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="J3" s="13" t="s">
+      <c r="K3" s="10" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="10">
-        <f>164+1</f>
-        <v>165</v>
-      </c>
-      <c r="C4" s="12">
+      <c r="B4" s="9">
+        <f>164</f>
+        <v>164</v>
+      </c>
+      <c r="C4" s="11">
         <f>B4/B6*100</f>
-        <v>93.75</v>
-      </c>
-      <c r="D4" s="10">
-        <f>99+1</f>
-        <v>100</v>
-      </c>
-      <c r="E4" s="12">
+        <v>93.714285714285722</v>
+      </c>
+      <c r="D4" s="9">
+        <v>107</v>
+      </c>
+      <c r="E4" s="11">
         <f>D4/D6*100</f>
-        <v>62.893081761006286</v>
-      </c>
-      <c r="F4" s="10">
+        <v>66.875</v>
+      </c>
+      <c r="F4" s="9">
         <f>B4+D4</f>
-        <v>265</v>
-      </c>
-      <c r="G4" s="12">
+        <v>271</v>
+      </c>
+      <c r="G4" s="11">
         <f>F4/F6*100</f>
-        <v>79.104477611940297</v>
-      </c>
-      <c r="I4" s="12">
-        <v>93.75</v>
-      </c>
-      <c r="J4" s="12">
-        <v>62.893081761006286</v>
+        <v>80.895522388059703</v>
+      </c>
+      <c r="J4" s="11">
+        <f>C4</f>
+        <v>93.714285714285722</v>
+      </c>
+      <c r="K4" s="11">
+        <f>E4</f>
+        <v>66.875</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="9">
         <v>11</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="11">
         <f>B5/B6*100</f>
-        <v>6.25</v>
-      </c>
-      <c r="D5" s="10">
-        <f>58+1</f>
-        <v>59</v>
-      </c>
-      <c r="E5" s="12">
+        <v>6.2857142857142865</v>
+      </c>
+      <c r="D5" s="9">
+        <f>53</f>
+        <v>53</v>
+      </c>
+      <c r="E5" s="11">
         <f>D5/D6*100</f>
-        <v>37.106918238993707</v>
-      </c>
-      <c r="F5" s="10">
+        <v>33.125</v>
+      </c>
+      <c r="F5" s="9">
         <f>B5+D5</f>
-        <v>70</v>
-      </c>
-      <c r="G5" s="12">
+        <v>64</v>
+      </c>
+      <c r="G5" s="11">
         <f>F5/F6*100</f>
-        <v>20.8955223880597</v>
-      </c>
-      <c r="I5" s="12">
-        <v>6.25</v>
-      </c>
-      <c r="J5" s="12">
-        <v>37.106918238993707</v>
+        <v>19.1044776119403</v>
+      </c>
+      <c r="J5" s="11">
+        <f>C5</f>
+        <v>6.2857142857142865</v>
+      </c>
+      <c r="K5" s="11">
+        <f>E5</f>
+        <v>33.125</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <f>SUM(B4:B5)</f>
-        <v>176</v>
-      </c>
-      <c r="C6" s="10">
+        <v>175</v>
+      </c>
+      <c r="C6" s="9">
         <f t="shared" ref="C6:G6" si="0">SUM(C4:C5)</f>
-        <v>100</v>
-      </c>
-      <c r="D6" s="10">
+        <v>100.00000000000001</v>
+      </c>
+      <c r="D6" s="9">
         <f t="shared" si="0"/>
-        <v>159</v>
-      </c>
-      <c r="E6" s="10">
+        <v>160</v>
+      </c>
+      <c r="E6" s="9">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="9">
         <f t="shared" si="0"/>
         <v>335</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="9">
         <f t="shared" si="0"/>
         <v>100</v>
       </c>
@@ -8562,13 +11970,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>27</v>
       </c>
@@ -8579,69 +11987,94 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="9">
         <v>31</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="11">
         <f>B2/B6*100</f>
         <v>34.831460674157306</v>
       </c>
+      <c r="F2" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="G2" s="11">
+        <v>34.831460674157306</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>25</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="11">
         <f>B3/B6*100</f>
         <v>28.08988764044944</v>
       </c>
+      <c r="F3" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="11">
+        <v>28.08988764044944</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>25</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="11">
         <f>B4/B6*100</f>
         <v>28.08988764044944</v>
       </c>
+      <c r="F4" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G4" s="11">
+        <v>28.08988764044944</v>
+      </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="9">
         <v>8</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="11">
         <f>B5/B6*100</f>
         <v>8.9887640449438209</v>
       </c>
+      <c r="F5" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G5" s="11">
+        <v>8.9887640449438209</v>
+      </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <f>SUM(B2:B5)</f>
         <v>89</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="9">
         <f>SUM(C2:C5)</f>
         <v>100</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -8650,14 +12083,14 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>42</v>
       </c>
@@ -8668,76 +12101,101 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="9">
         <v>31</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="11">
         <f>B2/B7*100</f>
         <v>34.831460674157306</v>
       </c>
+      <c r="F2" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="11">
+        <v>34.831460674157306</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>25</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="11">
         <f>B3/B7*100</f>
         <v>28.08988764044944</v>
       </c>
+      <c r="F3" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="11">
+        <v>28.08988764044944</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>25</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="11">
         <f>B4/B7*100</f>
         <v>28.08988764044944</v>
       </c>
+      <c r="F4" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="G4" s="11">
+        <v>28.08988764044944</v>
+      </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="9">
         <v>8</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="11">
         <f>B5/B7*100</f>
         <v>8.9887640449438209</v>
       </c>
+      <c r="F5" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="11">
+        <v>8.9887640449438209</v>
+      </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="10"/>
-      <c r="C6" s="12"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="11"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="10" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="9">
         <f>SUM(B2:B5)</f>
         <v>89</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <f>SUM(C2:C5)</f>
         <v>100</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -8747,93 +12205,93 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B2" s="10">
+      <c r="B2" s="9">
         <v>13</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="11">
         <f>B2/$B$7*100</f>
         <v>14.606741573033707</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="9">
         <v>52</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="11">
         <f t="shared" ref="C3:C6" si="0">B3/$B$7*100</f>
         <v>58.426966292134829</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="9">
         <v>0</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="9">
         <v>0</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="9">
         <v>24</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="11">
         <f t="shared" si="0"/>
         <v>26.966292134831459</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="10" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="9">
         <f>SUM(B2:B6)</f>
         <v>89</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="9">
         <f>SUM(C2:C6)</f>
         <v>100</v>
       </c>
@@ -8841,4 +12299,98 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A37B388-6521-440D-9FFB-5546F102E9EC}">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="9">
+        <v>6</v>
+      </c>
+      <c r="C2" s="11">
+        <f>B2/B5*100</f>
+        <v>6.7415730337078648</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="G2" s="11">
+        <v>6.7415730337078648</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="9">
+        <v>35</v>
+      </c>
+      <c r="C3" s="11">
+        <f>B3/B5*100</f>
+        <v>39.325842696629216</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" s="11">
+        <v>39.325842696629216</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="9">
+        <v>48</v>
+      </c>
+      <c r="C4" s="11">
+        <f>B4/B5*100</f>
+        <v>53.932584269662918</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="11">
+        <v>53.932584269662918</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="9">
+        <f>SUM(B2:B4)</f>
+        <v>89</v>
+      </c>
+      <c r="C5" s="9">
+        <f>SUM(C2:C4)</f>
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
continiue migration and estimate changed for quotation
</commit_message>
<xml_diff>
--- a/migration/tables.xlsx
+++ b/migration/tables.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\082_083\ward1\migration\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\migration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B656A17-B284-415C-AE49-C8DB0459A5C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA802FD1-DAF2-4FDD-8882-B4D5A2CBFC12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="8" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="10905" firstSheet="14" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Reasons for leaving origin" sheetId="1" r:id="rId1"/>
@@ -26,9 +26,11 @@
     <sheet name="Marrital status" sheetId="11" r:id="rId11"/>
     <sheet name="Family size" sheetId="12" r:id="rId12"/>
     <sheet name="dependency ratio" sheetId="13" r:id="rId13"/>
+    <sheet name="Leaving origin" sheetId="14" r:id="rId14"/>
+    <sheet name="Place of Origin" sheetId="15" r:id="rId15"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId14"/>
+    <externalReference r:id="rId16"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="98">
   <si>
     <t>2. Table No. 5.1.1: Distribution of Reasons for Leaving Place of Origin</t>
   </si>
@@ -320,6 +322,30 @@
   <si>
     <t>15-64</t>
   </si>
+  <si>
+    <t>Reasons for Left</t>
+  </si>
+  <si>
+    <t>Percentage</t>
+  </si>
+  <si>
+    <t>No/Limited opportunity</t>
+  </si>
+  <si>
+    <t>Unemployment</t>
+  </si>
+  <si>
+    <t>Political Instability</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>District</t>
+  </si>
+  <si>
+    <t>VDC/Municipality</t>
+  </si>
 </sst>
 </file>
 
@@ -461,7 +487,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -496,6 +522,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -511,9 +538,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2026,7 +2050,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -2152,7 +2176,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -13946,41 +13970,41 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:9" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
     </row>
-    <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
     </row>
-    <row r="3" spans="1:9" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -13991,7 +14015,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
@@ -14002,7 +14026,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
@@ -14013,7 +14037,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
@@ -14024,7 +14048,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
@@ -14035,7 +14059,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
@@ -14046,7 +14070,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>10</v>
       </c>
@@ -14057,7 +14081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>11</v>
       </c>
@@ -14068,7 +14092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>12</v>
       </c>
@@ -14092,35 +14116,35 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4681C5CD-AD1E-47C1-9DD5-E5803D1EB1C3}">
   <dimension ref="A1:I17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="6.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="18" t="s">
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="G1" s="19" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="19"/>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="20"/>
       <c r="B2" s="9" t="s">
         <v>36</v>
       </c>
@@ -14133,10 +14157,10 @@
       <c r="E2" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>57</v>
       </c>
@@ -14166,7 +14190,7 @@
         <v>2.8769707586578628</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
         <v>58</v>
       </c>
@@ -14196,7 +14220,7 @@
         <v>3.1532138525805147</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
         <v>59</v>
       </c>
@@ -14226,7 +14250,7 @@
         <v>7.2210618515024931</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="14" t="s">
         <v>60</v>
       </c>
@@ -14256,7 +14280,7 @@
         <v>4.9824821452634414</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
         <v>61</v>
       </c>
@@ -14286,7 +14310,7 @@
         <v>9.4882765125993807</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>62</v>
       </c>
@@ -14316,7 +14340,7 @@
         <v>8.7168171405470964</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
         <v>63</v>
       </c>
@@ -14346,7 +14370,7 @@
         <v>10.431545613798679</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
         <v>64</v>
       </c>
@@ -14376,7 +14400,7 @@
         <v>8.497843956340116</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>65</v>
       </c>
@@ -14406,7 +14430,7 @@
         <v>9.7173561514620665</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>66</v>
       </c>
@@ -14436,7 +14460,7 @@
         <v>7.6876431747742888</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>67</v>
       </c>
@@ -14466,7 +14490,7 @@
         <v>8.8027220051206037</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>68</v>
       </c>
@@ -14496,7 +14520,7 @@
         <v>8.0784260881282837</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>69</v>
       </c>
@@ -14526,7 +14550,7 @@
         <v>3.6770650855679827</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>70</v>
       </c>
@@ -14556,7 +14580,7 @@
         <v>6.6685756636571893</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>12</v>
       </c>
@@ -14597,48 +14621,48 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5FC4570-8427-483C-9157-77FE223CE978}">
   <dimension ref="A1:O7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.6640625" customWidth="1"/>
-    <col min="13" max="13" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.7109375" customWidth="1"/>
+    <col min="13" max="13" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="18" t="s">
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="18"/>
+      <c r="G1" s="19"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A2" s="19"/>
-      <c r="B2" s="20" t="s">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" s="20"/>
+      <c r="B2" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20" t="s">
+      <c r="C2" s="21"/>
+      <c r="D2" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="20"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
       <c r="N2" t="s">
         <v>77</v>
       </c>
@@ -14646,8 +14670,8 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A3" s="19"/>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" s="20"/>
       <c r="B3" s="9" t="s">
         <v>74</v>
       </c>
@@ -14678,7 +14702,7 @@
         <v>34.615384615384613</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>75</v>
       </c>
@@ -14726,7 +14750,7 @@
         <v>65.384615384615387</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>76</v>
       </c>
@@ -14735,7 +14759,7 @@
         <v>99</v>
       </c>
       <c r="C5" s="11">
-        <f t="shared" ref="C5:C6" si="0">B5/$B$6*100</f>
+        <f t="shared" ref="C5" si="0">B5/$B$6*100</f>
         <v>58.928571428571431</v>
       </c>
       <c r="D5" s="9">
@@ -14763,7 +14787,7 @@
         <v>62.037037037037038</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -14791,12 +14815,10 @@
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="J6" s="21"/>
-      <c r="K6" s="22"/>
+      <c r="K6" s="13"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="J7" s="21"/>
-      <c r="K7" s="22"/>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K7" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -14815,14 +14837,14 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3986BFF3-A766-496C-9200-083AC941658F}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>82</v>
       </c>
@@ -14833,7 +14855,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>79</v>
       </c>
@@ -14852,8 +14874,8 @@
         <v>77.528089887640448</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="23" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="16" t="s">
         <v>80</v>
       </c>
       <c r="B3" s="9">
@@ -14863,15 +14885,15 @@
         <f t="shared" ref="C3:C5" si="0">B3/$B$5*100</f>
         <v>16.853932584269664</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" s="16" t="s">
         <v>80</v>
       </c>
       <c r="G3" s="11">
-        <f t="shared" ref="G3:G5" si="1">C3</f>
+        <f t="shared" ref="G3:G4" si="1">C3</f>
         <v>16.853932584269664</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>81</v>
       </c>
@@ -14890,7 +14912,7 @@
         <v>5.6179775280898872</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>12</v>
       </c>
@@ -14914,12 +14936,12 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC3014F1-1703-47D5-A2CD-2B891BFB9566}">
   <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>83</v>
       </c>
@@ -14943,7 +14965,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>84</v>
       </c>
@@ -14973,7 +14995,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>85</v>
       </c>
@@ -15003,7 +15025,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>12</v>
       </c>
@@ -15039,50 +15061,165 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDF745B5-F0A4-4C32-BF38-D8BF1F0ED0B6}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E211E5C9-7DF2-4829-BE18-8FD1E5D07B3F}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:12" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
     </row>
-    <row r="2" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:12" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>15</v>
       </c>
@@ -15093,7 +15230,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>16</v>
       </c>
@@ -15104,7 +15241,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>17</v>
       </c>
@@ -15115,7 +15252,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>18</v>
       </c>
@@ -15126,7 +15263,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -15150,46 +15287,46 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.109375" customWidth="1"/>
+    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:11" ht="20.25" x14ac:dyDescent="0.25">
+      <c r="A1" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
     </row>
-    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
     </row>
-    <row r="3" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>21</v>
       </c>
@@ -15200,7 +15337,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
@@ -15211,7 +15348,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>23</v>
       </c>
@@ -15222,7 +15359,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>24</v>
       </c>
@@ -15233,7 +15370,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
@@ -15257,12 +15394,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>25</v>
       </c>
@@ -15270,7 +15407,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>2083</v>
       </c>
@@ -15278,7 +15415,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="9">
         <v>2082</v>
       </c>
@@ -15286,7 +15423,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>2081</v>
       </c>
@@ -15294,7 +15431,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
         <v>2080</v>
       </c>
@@ -15302,7 +15439,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>2079</v>
       </c>
@@ -15310,7 +15447,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
         <v>2078</v>
       </c>
@@ -15318,7 +15455,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
         <v>2077</v>
       </c>
@@ -15326,7 +15463,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
         <v>2076</v>
       </c>
@@ -15334,7 +15471,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
         <v>2075</v>
       </c>
@@ -15342,7 +15479,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
         <v>2074</v>
       </c>
@@ -15350,7 +15487,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>12</v>
       </c>
@@ -15368,38 +15505,38 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="19" t="s">
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="19"/>
+      <c r="G1" s="20"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="19"/>
-      <c r="B2" s="18" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="20"/>
+      <c r="B2" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18" t="s">
+      <c r="C2" s="19"/>
+      <c r="D2" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="E2" s="18"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="19"/>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="20"/>
       <c r="B3" s="10" t="s">
         <v>37</v>
       </c>
@@ -15425,7 +15562,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>38</v>
       </c>
@@ -15461,7 +15598,7 @@
         <v>66.875</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>39</v>
       </c>
@@ -15497,7 +15634,7 @@
         <v>33.125</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -15542,12 +15679,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>27</v>
       </c>
@@ -15558,7 +15695,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>30</v>
       </c>
@@ -15578,7 +15715,7 @@
         <v>31.460674157303369</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>31</v>
       </c>
@@ -15598,7 +15735,7 @@
         <v>35.955056179775283</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>40</v>
       </c>
@@ -15618,7 +15755,7 @@
         <v>25.842696629213485</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>41</v>
       </c>
@@ -15638,7 +15775,7 @@
         <v>6.7415730337078648</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -15664,13 +15801,13 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>42</v>
       </c>
@@ -15681,7 +15818,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>43</v>
       </c>
@@ -15701,7 +15838,7 @@
         <v>67.415730337078656</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>44</v>
       </c>
@@ -15721,7 +15858,7 @@
         <v>25.842696629213485</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>45</v>
       </c>
@@ -15740,7 +15877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>46</v>
       </c>
@@ -15760,7 +15897,7 @@
         <v>6.7415730337078648</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>12</v>
       </c>
@@ -15786,14 +15923,14 @@
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>47</v>
       </c>
@@ -15804,7 +15941,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>49</v>
       </c>
@@ -15817,7 +15954,7 @@
         <v>17.977528089887642</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>50</v>
       </c>
@@ -15830,7 +15967,7 @@
         <v>69.662921348314612</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>51</v>
       </c>
@@ -15842,7 +15979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>52</v>
       </c>
@@ -15854,7 +15991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>32</v>
       </c>
@@ -15866,7 +16003,7 @@
         <v>12.359550561797752</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
         <v>12</v>
       </c>
@@ -15888,14 +16025,14 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A37B388-6521-440D-9FFB-5546F102E9EC}">
   <dimension ref="A1:G5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>53</v>
       </c>
@@ -15906,7 +16043,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>54</v>
       </c>
@@ -15925,7 +16062,7 @@
         <v>53.932584269662918</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>56</v>
       </c>
@@ -15944,7 +16081,7 @@
         <v>39.325842696629216</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>55</v>
       </c>
@@ -15963,7 +16100,7 @@
         <v>6.7415730337078648</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>12</v>
       </c>

</xml_diff>